<commit_message>
Finalize V1.6.6 conversational spare inventory mutation
</commit_message>
<xml_diff>
--- a/database/spares/critical_spares.xlsx
+++ b/database/spares/critical_spares.xlsx
@@ -9360,7 +9360,7 @@
         </is>
       </c>
       <c r="I9" s="247" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J9" s="247" t="n">
         <v>0</v>
@@ -11766,7 +11766,7 @@
         </is>
       </c>
       <c r="G3" s="263" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H3" s="263" t="n">
         <v>1</v>
@@ -13785,7 +13785,7 @@
         </is>
       </c>
       <c r="G2" s="146" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H2" s="146" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
ANVIQO V1.0 release gate and production deployment
</commit_message>
<xml_diff>
--- a/database/spares/critical_spares.xlsx
+++ b/database/spares/critical_spares.xlsx
@@ -8876,6 +8876,7 @@
     <mergeCell ref="I2:I4"/>
     <mergeCell ref="M5:M7"/>
     <mergeCell ref="N5:N7"/>
+    <mergeCell ref="B5:B7"/>
     <mergeCell ref="J5:J7"/>
     <mergeCell ref="D5:D7"/>
     <mergeCell ref="C2:C4"/>
@@ -8884,12 +8885,11 @@
     <mergeCell ref="C5:C7"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="K5:K7"/>
-    <mergeCell ref="B2:B4"/>
     <mergeCell ref="F5:F7"/>
     <mergeCell ref="L5:L7"/>
     <mergeCell ref="D2:D4"/>
     <mergeCell ref="O5:O7"/>
-    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B2:B4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" scale="76"/>
@@ -9360,7 +9360,7 @@
         </is>
       </c>
       <c r="I9" s="247" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J9" s="247" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Finalize ANVIQO critical spare intelligence and routing
</commit_message>
<xml_diff>
--- a/database/spares/critical_spares.xlsx
+++ b/database/spares/critical_spares.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="RTD" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="LT" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="PT" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="FT" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="MCV" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FSV&amp;PCV" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="SOV" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="POS'R" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="LOAD CELL" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Analyser" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Sheet1" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="AIR COMPRESSOR" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Sheet2" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTD" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LT" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PT" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FT" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCV" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FSV&amp;PCV" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOV" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POS'R" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LOAD CELL" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analyser" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AIR COMPRESSOR" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'LT'!$A$1:$O$9</definedName>
@@ -8876,7 +8876,6 @@
     <mergeCell ref="I2:I4"/>
     <mergeCell ref="M5:M7"/>
     <mergeCell ref="N5:N7"/>
-    <mergeCell ref="B5:B7"/>
     <mergeCell ref="J5:J7"/>
     <mergeCell ref="D5:D7"/>
     <mergeCell ref="C2:C4"/>
@@ -8884,12 +8883,13 @@
     <mergeCell ref="J2:J4"/>
     <mergeCell ref="C5:C7"/>
     <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B2:B4"/>
     <mergeCell ref="K5:K7"/>
     <mergeCell ref="F5:F7"/>
     <mergeCell ref="L5:L7"/>
     <mergeCell ref="D2:D4"/>
     <mergeCell ref="O5:O7"/>
-    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B5:B7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" scale="76"/>

</xml_diff>